<commit_message>
feat: complete Power Query ETL practice with data cleaning and transformation
</commit_message>
<xml_diff>
--- a/01_excel/02_formulas_repaso/repaso_formulas.xlsx
+++ b/01_excel/02_formulas_repaso/repaso_formulas.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmnav\Documents\Data_Analytics\data-analytics-portfolio\01_excel\02_formulas_repaso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F409F59-AC74-4983-B865-7452A776C3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{957D5551-CAA3-42F9-9600-3A6A6945EBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{867C6D99-EF6E-4239-A5C9-FB9EA77BB38E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Repaso" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>